<commit_message>
Add usage data for 23 Oct 2026 (7 logins); merge 3 late 22 Oct logins
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/daily_snapshots/Daily Usage Snapshot - 22-10-2026.xlsx
+++ b/daily_snapshots/Daily Usage Snapshot - 22-10-2026.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -980,6 +980,147 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>user1792679878.2725</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ciara@the-ear.co.uk</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ciara</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Ciara@the-ear.co.uk</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>School Administrator</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Thursday, 22 October 2026 at 18:26</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>York High School</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Classroom</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Paying</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>user1788779472.8089</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>samanthanel@icloud.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pieter-Willem</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Nel</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Participant</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Thursday, 22 October 2026 at 17:48</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Educ8sa</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Instrumental</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Paying</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>user1761656532.9835</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hummingbirds@generationschools.co.za</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Octavia</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Josephs</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Teacher</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Thursday, 22 October 2026 at 16:30</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Generation Schools Hermanus</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Classroom</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Paying</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>